<commit_message>
Actualización automática 2026-09-17 10:30:17
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:R38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FERRETERIA Y MADERAS S.A. MADEFER</t>
+          <t>FLORES PARRA CLEIVER YOEL</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>FLORES PARRA CLEIVER YOEL</t>
+          <t>GRATEROL CASTILLO STEFFANY PAOLA ROSDALY</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GRATEROL CASTILLO STEFFANY PAOLA ROSDALY</t>
+          <t>GUILLEN PARRALES KATERINE MABEL</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GUILLEN PARRALES KATERINE MABEL</t>
+          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
+          <t>IMPORTELECTRIC S.A.S</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IMPORTELECTRIC S.A.S</t>
+          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
+          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
+          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
+          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>0</v>
+        <v>37.08</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
+          <t>LUI WONG ANGEL BOLIVAR</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2280,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="M30" s="2" t="n">
-        <v>37.08</v>
+        <v>0</v>
       </c>
       <c r="N30" s="2" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>LUI WONG ANGEL BOLIVAR</t>
+          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
+          <t>PUCO TOAPANTA MARCO ANTONIO</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PUCO TOAPANTA MARCO ANTONIO</t>
+          <t>SANCHEZ BAJANA FRAK XAVIER</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SANCHEZ BAJANA FRAK XAVIER</t>
+          <t>SANCHEZ CORREA WILSON SERGIO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SANCHEZ CORREA WILSON SERGIO</t>
+          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2565,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I35" s="2" t="n">
         <v>0</v>
@@ -2577,10 +2577,10 @@
         <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>0</v>
+        <v>479.69</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>0</v>
+        <v>1344.33</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
+          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2625,7 +2625,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="I36" s="2" t="n">
         <v>0</v>
@@ -2637,10 +2637,10 @@
         <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
-        <v>479.69</v>
+        <v>0</v>
       </c>
       <c r="M36" s="2" t="n">
-        <v>1344.33</v>
+        <v>0</v>
       </c>
       <c r="N36" s="2" t="n">
         <v>0</v>
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
+          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2719,144 +2719,84 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R38" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>1 de 37</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>1 de 37</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>1 de 37</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>1 de 37</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="L39" s="4" t="inlineStr">
-        <is>
-          <t>1 de 37</t>
-        </is>
-      </c>
-      <c r="M39" s="4" t="inlineStr">
-        <is>
-          <t>4 de 37</t>
-        </is>
-      </c>
-      <c r="N39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="P39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="Q39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
-        </is>
-      </c>
-      <c r="R39" s="4" t="inlineStr">
-        <is>
-          <t>0 de 37</t>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>1 de 36</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>1 de 36</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>1 de 36</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>1 de 36</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>1 de 36</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>4 de 36</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
+        </is>
+      </c>
+      <c r="R38" s="4" t="inlineStr">
+        <is>
+          <t>0 de 36</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3360,14 +3300,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FERRETERIA Y MADERAS S.A. MADEFER</t>
+          <t>FLORES PARRA CLEIVER YOEL</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>8681.9</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>0</v>
+        <v>5421.72</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -3376,7 +3316,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="19">
@@ -3387,14 +3327,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>FLORES PARRA CLEIVER YOEL</t>
+          <t>GUILLEN PARRALES KATERINE MABEL</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>8681.9</v>
+        <v>204.88</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>5421.72</v>
+        <v>109.48</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -3403,7 +3343,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="20">
@@ -3414,14 +3354,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GUILLEN PARRALES KATERINE MABEL</t>
+          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>204.88</v>
+        <v>7835.2</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>109.48</v>
+        <v>0</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>0</v>
@@ -3430,7 +3370,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="21">
@@ -3441,11 +3381,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
+          <t>IMPORTELECTRIC S.A.S</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>7835.2</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>0</v>
@@ -3457,7 +3397,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3468,14 +3408,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>IMPORTELECTRIC S.A.S</t>
+          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>0</v>
+        <v>2493.92</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -3484,7 +3424,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="23">
@@ -3495,14 +3435,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
+          <t>INTROMEX S.A.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>2493.92</v>
+        <v>0</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>0</v>
@@ -3511,7 +3451,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -3522,7 +3462,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>INTROMEX S.A.</t>
+          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -3549,7 +3489,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
+          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -3576,7 +3516,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
+          <t>LUI WONG ANGEL BOLIVAR</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -3603,23 +3543,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LUI WONG ANGEL BOLIVAR</t>
+          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0</v>
+        <v>1327.27</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0</v>
+        <v>270.66</v>
       </c>
       <c r="F27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="28">
@@ -3630,23 +3570,23 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
+          <t>PUCO TOAPANTA MARCO ANTONIO</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1327.27</v>
+        <v>0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>270.66</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3657,7 +3597,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PUCO TOAPANTA MARCO ANTONIO</t>
+          <t>RODRIGUEZ PAILACHO VICENTE JONY</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -3673,7 +3613,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="30">
@@ -3684,7 +3624,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RODRIGUEZ PAILACHO VICENTE JONY</t>
+          <t>SANCHEZ BAJANA FRAK XAVIER</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -3700,7 +3640,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -3711,7 +3651,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SANCHEZ BAJANA FRAK XAVIER</t>
+          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -3721,56 +3661,29 @@
         <v>0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0</v>
+        <v>2127.79</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0</v>
+        <v>2606.12</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>2127.79</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>2606.12</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="C33" s="6" t="n">
+      <c r="C32" s="6" t="n">
         <v>37855.35</v>
       </c>
-      <c r="D33" s="6" t="n">
+      <c r="D32" s="6" t="n">
         <v>40935.59</v>
       </c>
-      <c r="E33" s="6" t="n">
+      <c r="E32" s="6" t="n">
         <v>39346.94</v>
       </c>
-      <c r="F33" s="6" t="n">
+      <c r="F32" s="6" t="n">
         <v>9974.860000000001</v>
       </c>
-      <c r="G33" s="6" t="n">
+      <c r="G32" s="6" t="n">
         <v>39500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización automática 2026-09-21 17:30:18
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -2325,10 +2325,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0</v>
+        <v>313.2</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0</v>
+        <v>178.42</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0</v>
@@ -2568,7 +2568,7 @@
         <v>782.1</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0</v>
+        <v>206.29</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
@@ -2746,12 +2746,12 @@
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>1 de 36</t>
+          <t>2 de 36</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>1 de 36</t>
+          <t>3 de 36</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3016,7 +3016,7 @@
         <v>22863.45</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>49.75</v>
+        <v>1286.98</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>8000</v>
@@ -3556,7 +3556,7 @@
         <v>270.66</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0</v>
+        <v>491.62</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>2000</v>
@@ -3664,7 +3664,7 @@
         <v>2127.79</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>2606.12</v>
+        <v>2812.41</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>2000</v>
@@ -3681,7 +3681,7 @@
         <v>39346.94</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>12042.59</v>
+        <v>13977.73</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>39500</v>
@@ -3804,13 +3804,13 @@
         <v>3635</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0</v>
+        <v>1237.23</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3635</v>
+        <v>2397.77</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>0.3403658872077029</v>
       </c>
     </row>
     <row r="5">
@@ -3876,13 +3876,13 @@
         <v>615</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>782.1</v>
+        <v>1095.3</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-167.1</v>
+        <v>-480.3</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.271707317073171</v>
+        <v>1.780975609756098</v>
       </c>
     </row>
     <row r="8">
@@ -3900,13 +3900,13 @@
         <v>463</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>2295.28</v>
+        <v>2679.99</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-1832.28</v>
+        <v>-2216.99</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>4.957408207343413</v>
+        <v>5.788315334773218</v>
       </c>
     </row>
     <row r="9">
@@ -4087,13 +4087,13 @@
         <v>45197.643</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>12083.73</v>
+        <v>14018.87</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>33113.913</v>
+        <v>31178.773</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2673531006915559</v>
+        <v>0.3101681651850739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-22 08:30:17
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>-54.81</v>
+        <v>1973.38</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>4 de 36</t>
+          <t>5 de 36</t>
         </is>
       </c>
       <c r="N38" s="4" t="inlineStr">
@@ -3016,7 +3016,7 @@
         <v>22863.45</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1286.98</v>
+        <v>3315.17</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>8000</v>
@@ -3681,7 +3681,7 @@
         <v>39346.94</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>13977.73</v>
+        <v>16005.92</v>
       </c>
       <c r="G32" s="6" t="n">
         <v>39500</v>
@@ -3704,7 +3704,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -4044,13 +4044,13 @@
         <v>35464</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8011.82</v>
+        <v>10040.01</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>27452.18</v>
+        <v>25423.99</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2259141664786826</v>
+        <v>0.2831042747575006</v>
       </c>
     </row>
     <row r="15">
@@ -4087,13 +4087,13 @@
         <v>45197.643</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>14018.87</v>
+        <v>16047.06</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>31178.773</v>
+        <v>29150.583</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3101681651850739</v>
+        <v>0.3550419653520428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-25 11:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R38"/>
+  <dimension ref="A1:R37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COMISARIATO DEL CONSTRUCTOR COMITRUCTOR S.A.</t>
+          <t>CONTRATISTAS ACABADOS PARA LA CONTRUCCION JANDRI S.A.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CONTRATISTAS ACABADOS PARA LA CONTRUCCION JANDRI S.A.</t>
+          <t>COZZARELLI CONTRERAS FATIMA MERCEDES</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>COZZARELLI CONTRERAS FATIMA MERCEDES</t>
+          <t>DEPODECON S.A.</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DEPODECON S.A.</t>
+          <t>DISTRIBUIDORA Y SERVICIOS ELÉCTRICOS  ELEKTRICELL S.A.</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA Y SERVICIOS ELÉCTRICOS  ELEKTRICELL S.A.</t>
+          <t>ELECTROKOLER S.A.</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ELECTROKOLER S.A.</t>
+          <t>FLORES PARRA CLEIVER YOEL</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FLORES PARRA CLEIVER YOEL</t>
+          <t>GRATEROL CASTILLO STEFFANY PAOLA ROSDALY</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1766,7 +1766,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>GRATEROL CASTILLO STEFFANY PAOLA ROSDALY</t>
+          <t>GUILLEN PARRALES KATERINE MABEL</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GUILLEN PARRALES KATERINE MABEL</t>
+          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
+          <t>IMPORTELECTRIC S.A.S</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>IMPORTELECTRIC S.A.S</t>
+          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
+          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
+          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
+          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2160,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>37.08</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
+          <t>LUI WONG ANGEL BOLIVAR</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -2220,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>37.08</v>
+        <v>0</v>
       </c>
       <c r="N29" s="2" t="n">
         <v>0</v>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>LUI WONG ANGEL BOLIVAR</t>
+          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -2265,10 +2265,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0</v>
+        <v>313.2</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0</v>
+        <v>178.42</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0</v>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
+          <t>PUCO TOAPANTA MARCO ANTONIO</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -2325,10 +2325,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>313.2</v>
+        <v>0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>178.42</v>
+        <v>0</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0</v>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>PUCO TOAPANTA MARCO ANTONIO</t>
+          <t>SANCHEZ BAJANA FRAK XAVIER</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SANCHEZ BAJANA FRAK XAVIER</t>
+          <t>SANCHEZ CORREA WILSON SERGIO</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SANCHEZ CORREA WILSON SERGIO</t>
+          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -2505,10 +2505,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0</v>
+        <v>782.1</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0</v>
+        <v>206.29</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0</v>
@@ -2517,10 +2517,10 @@
         <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
-        <v>0</v>
+        <v>479.69</v>
       </c>
       <c r="M34" s="2" t="n">
-        <v>0</v>
+        <v>1344.33</v>
       </c>
       <c r="N34" s="2" t="n">
         <v>0</v>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
+          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2565,10 +2565,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>782.1</v>
+        <v>0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>206.29</v>
+        <v>0</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0</v>
@@ -2577,10 +2577,10 @@
         <v>0</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>479.69</v>
+        <v>0</v>
       </c>
       <c r="M35" s="2" t="n">
-        <v>1344.33</v>
+        <v>0</v>
       </c>
       <c r="N35" s="2" t="n">
         <v>0</v>
@@ -2606,7 +2606,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SORIA AVELLAN RAFAEL HUMBERTO</t>
+          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -2659,144 +2659,84 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>SOTOMAYOR ORTIZ LUIS JAVIER</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>1 de 36</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>1 de 36</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>2 de 36</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>3 de 36</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>1 de 36</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="L38" s="4" t="inlineStr">
-        <is>
-          <t>1 de 36</t>
-        </is>
-      </c>
-      <c r="M38" s="4" t="inlineStr">
-        <is>
-          <t>5 de 36</t>
-        </is>
-      </c>
-      <c r="N38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="P38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="Q38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
-        </is>
-      </c>
-      <c r="R38" s="4" t="inlineStr">
-        <is>
-          <t>0 de 36</t>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>1 de 35</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>1 de 35</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>2 de 35</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>3 de 35</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>1 de 35</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>1 de 35</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>5 de 35</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="P37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="Q37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
+        </is>
+      </c>
+      <c r="R37" s="4" t="inlineStr">
+        <is>
+          <t>0 de 35</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3165,7 +3105,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>COMISARIATO DEL CONSTRUCTOR COMITRUCTOR S.A.</t>
+          <t>CONTRATISTAS ACABADOS PARA LA CONTRUCCION JANDRI S.A.</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -3175,13 +3115,13 @@
         <v>0</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>507.91</v>
+        <v>0</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3192,7 +3132,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CONTRATISTAS ACABADOS PARA LA CONTRUCCION JANDRI S.A.</t>
+          <t>DEPODECON S.A.</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -3219,7 +3159,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DEPODECON S.A.</t>
+          <t>DISTRIBUIDORA Y SERVICIOS ELÉCTRICOS  ELEKTRICELL S.A.</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -3246,7 +3186,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DISTRIBUIDORA Y SERVICIOS ELÉCTRICOS  ELEKTRICELL S.A.</t>
+          <t>ELECTROKOLER S.A.</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -3273,14 +3213,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ELECTROKOLER S.A.</t>
+          <t>FLORES PARRA CLEIVER YOEL</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0</v>
+        <v>8681.9</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>0</v>
+        <v>5421.72</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>0</v>
@@ -3289,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>0</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="18">
@@ -3300,14 +3240,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>FLORES PARRA CLEIVER YOEL</t>
+          <t>GUILLEN PARRALES KATERINE MABEL</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>8681.9</v>
+        <v>204.88</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>5421.72</v>
+        <v>109.48</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>0</v>
@@ -3316,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="19">
@@ -3327,14 +3267,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>GUILLEN PARRALES KATERINE MABEL</t>
+          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>204.88</v>
+        <v>7835.2</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>109.48</v>
+        <v>0</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>0</v>
@@ -3343,7 +3283,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>1000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="20">
@@ -3354,11 +3294,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>GUZMAN MAYORGA ROMINA SISNEY</t>
+          <t>IMPORTELECTRIC S.A.S</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7835.2</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
         <v>0</v>
@@ -3370,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -3381,14 +3321,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>IMPORTELECTRIC S.A.S</t>
+          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0</v>
+        <v>2493.92</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>0</v>
@@ -3397,7 +3337,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -3408,14 +3348,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>INTERNEGOCIOS DE HIERRO S.A.</t>
+          <t>INTROMEX S.A.</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>2493.92</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>0</v>
@@ -3424,7 +3364,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -3435,7 +3375,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>INTROMEX S.A.</t>
+          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -3462,7 +3402,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ITURRALDE ROSALES FRANKLIN DAVID</t>
+          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -3489,7 +3429,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LINDAO MEJIA FERNANDO AGUILUCHO</t>
+          <t>LUI WONG ANGEL BOLIVAR</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -3516,23 +3456,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LUI WONG ANGEL BOLIVAR</t>
+          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>0</v>
+        <v>1327.27</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0</v>
+        <v>270.66</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>491.62</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="27">
@@ -3543,23 +3483,23 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MUÑOZ FALCONES SERGIO BACILIO</t>
+          <t>PUCO TOAPANTA MARCO ANTONIO</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1327.27</v>
+        <v>0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>270.66</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>491.62</v>
+        <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3570,7 +3510,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PUCO TOAPANTA MARCO ANTONIO</t>
+          <t>RODRIGUEZ PAILACHO VICENTE JONY</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -3586,7 +3526,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="29">
@@ -3597,7 +3537,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RODRIGUEZ PAILACHO VICENTE JONY</t>
+          <t>SANCHEZ BAJANA FRAK XAVIER</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -3613,7 +3553,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -3624,7 +3564,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SANCHEZ BAJANA FRAK XAVIER</t>
+          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -3634,57 +3574,30 @@
         <v>0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0</v>
+        <v>2127.79</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>2812.41</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>LINDAO ZUÑIGA BRYAN JOSE</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>SOCIEDAD CIVIL Y COMERCIAL GRUPO MOLINA PROAÑO</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>2127.79</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>2812.41</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32" s="6" t="n">
+      <c r="C31" s="6" t="n">
         <v>37855.35</v>
       </c>
-      <c r="D32" s="6" t="n">
+      <c r="D31" s="6" t="n">
         <v>40935.59</v>
       </c>
-      <c r="E32" s="6" t="n">
-        <v>39346.94</v>
-      </c>
-      <c r="F32" s="6" t="n">
+      <c r="E31" s="6" t="n">
+        <v>38839.03</v>
+      </c>
+      <c r="F31" s="6" t="n">
         <v>31534.27</v>
       </c>
-      <c r="G32" s="6" t="n">
-        <v>39500</v>
+      <c r="G31" s="6" t="n">
+        <v>38500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-07 12:51:42
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -2851,7 +2851,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>1500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="4">
@@ -2905,7 +2905,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="6">
@@ -2932,7 +2932,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -2959,7 +2959,7 @@
         <v>-30.93</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>8000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="8">
@@ -3013,7 +3013,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="10">
@@ -3040,7 +3040,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -3067,7 +3067,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="12">
@@ -3094,7 +3094,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="13">
@@ -3229,7 +3229,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
     </row>
     <row r="19">
@@ -3283,7 +3283,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="20">
@@ -3337,7 +3337,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>1500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -3472,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>2000</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="27">
@@ -3526,7 +3526,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -3580,7 +3580,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="31">
@@ -3597,7 +3597,7 @@
         <v>-30.93</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>38500</v>
+        <v>45800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-15 17:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1263,7 +1263,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0</v>
+        <v>3425.19</v>
       </c>
       <c r="O13" s="2" t="n">
         <v>0</v>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="N37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>1 de 35</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
@@ -3091,7 +3091,7 @@
         <v>7218.83</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>3425.19</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -3594,7 +3594,7 @@
         <v>46838.78</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>14817.41</v>
+        <v>18242.6</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>45800</v>
@@ -3981,13 +3981,13 @@
         <v>1198.8</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0</v>
+        <v>3425.19</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>1198.8</v>
+        <v>-2226.39</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>2.857182182182182</v>
       </c>
     </row>
     <row r="16">
@@ -4000,13 +4000,13 @@
         <v>45770.97300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>14817.41</v>
+        <v>18242.6</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>30953.563</v>
+        <v>27528.373</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3237294081556885</v>
+        <v>0.3985626436213186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-16 17:30:18
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -2160,7 +2160,7 @@
         <v>0</v>
       </c>
       <c r="M28" s="2" t="n">
-        <v>0</v>
+        <v>67.39</v>
       </c>
       <c r="N28" s="2" t="n">
         <v>0</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>1 de 35</t>
+          <t>2 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -3957,13 +3957,13 @@
         <v>36800.33</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13628.62</v>
+        <v>13696.01</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>23171.71</v>
+        <v>23104.32</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3703396138023762</v>
+        <v>0.3721708473809882</v>
       </c>
     </row>
     <row r="15">
@@ -4000,13 +4000,13 @@
         <v>45770.97300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>18242.6</v>
+        <v>18309.99</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>27528.373</v>
+        <v>27460.983</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3985626436213186</v>
+        <v>0.4000349741308754</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-22 15:30:19
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>1219.72</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13628.62</v>
+        <v>13591.68</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2956,7 +2956,7 @@
         <v>27556.24</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>14817.41</v>
+        <v>14780.47</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>30000</v>
@@ -3594,7 +3594,7 @@
         <v>46838.78</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>18242.6</v>
+        <v>18205.66</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>45800</v>
@@ -3957,13 +3957,13 @@
         <v>36800.33</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13696.01</v>
+        <v>13659.07</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>23104.32</v>
+        <v>23141.26</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3721708473809882</v>
+        <v>0.3711670520345877</v>
       </c>
     </row>
     <row r="15">
@@ -4000,13 +4000,13 @@
         <v>45770.97300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>18309.99</v>
+        <v>18273.05</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>27460.983</v>
+        <v>27497.923</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.4000349741308754</v>
+        <v>0.3992279124151457</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-27 17:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -900,7 +900,7 @@
         <v>1219.72</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>13523.57</v>
+        <v>23368.67</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -2514,7 +2514,7 @@
         <v>0</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>0</v>
+        <v>710.64</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2701,7 +2701,7 @@
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>0 de 35</t>
+          <t>1 de 35</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
@@ -2956,7 +2956,7 @@
         <v>27556.24</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>14712.36</v>
+        <v>24557.46</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>30000</v>
@@ -3469,7 +3469,7 @@
         <v>491.62</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>0</v>
+        <v>446.04</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>1800</v>
@@ -3577,7 +3577,7 @@
         <v>2786.39</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>0</v>
+        <v>710.64</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>1500</v>
@@ -3594,7 +3594,7 @@
         <v>46838.78</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>18137.55</v>
+        <v>29139.33</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>45800</v>
@@ -3618,7 +3618,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3885,13 +3885,13 @@
         <v>203.763</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>710.64</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>203.763</v>
+        <v>-506.877</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>3.487581160465835</v>
       </c>
     </row>
     <row r="12">
@@ -3909,13 +3909,13 @@
         <v>350</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>446.04</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>350</v>
+        <v>-96.04000000000002</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>1.2744</v>
       </c>
     </row>
     <row r="13">
@@ -3957,13 +3957,13 @@
         <v>36800.33</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>13590.96</v>
+        <v>23436.06</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>23209.37</v>
+        <v>13364.27</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.3693162534140318</v>
+        <v>0.6368437456946717</v>
       </c>
     </row>
     <row r="15">
@@ -4000,13 +4000,13 @@
         <v>45770.97300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>18204.94</v>
+        <v>29206.72</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>27566.033</v>
+        <v>16564.253</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3977398514119417</v>
+        <v>0.6381057269636806</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 09:30:16
</commit_message>
<xml_diff>
--- a/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
+++ b/data/LINDAO ZUÑIGA BRYAN JOSE.xlsx
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>1514.84</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>3425.19</v>
@@ -2711,7 +2711,7 @@
       </c>
       <c r="M37" s="4" t="inlineStr">
         <is>
-          <t>2 de 35</t>
+          <t>3 de 35</t>
         </is>
       </c>
       <c r="N37" s="4" t="inlineStr">
@@ -3091,7 +3091,7 @@
         <v>7218.83</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3425.19</v>
+        <v>4940.03</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>2000</v>
@@ -3594,7 +3594,7 @@
         <v>46838.78</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>29139.33</v>
+        <v>30654.17</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>45800</v>
@@ -3617,7 +3617,7 @@
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3957,13 +3957,13 @@
         <v>36800.33</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>23436.06</v>
+        <v>24950.9</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>13364.27</v>
+        <v>11849.43</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.6368437456946717</v>
+        <v>0.6780075069978992</v>
       </c>
     </row>
     <row r="15">
@@ -4000,13 +4000,13 @@
         <v>45770.97300000001</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>29206.72</v>
+        <v>30721.56</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>16564.253</v>
+        <v>15049.413</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.6381057269636806</v>
+        <v>0.6712018116809533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>